<commit_message>
Add the Alera voice script as a Word file and capitalize patient replies.
The Evolve build sheet lists every voice question, bucket, and configured line. SMS demo replies now start with a capital letter.

Co-authored-by: kiannuzzi-byte <kiannuzzi-byte@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Alera-IBHH-Enrollment-SMS.xlsx
+++ b/Alera-IBHH-Enrollment-SMS.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="template" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="template" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -464,7 +464,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>yes who is this</t>
+          <t>Yes who is this</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -500,7 +500,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>is this a scam lol</t>
+          <t>Is this a scam lol</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -522,7 +522,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>i got a letter about medicaid changing and im worried</t>
+          <t>I got a letter about Medicaid changing and I'm worried</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -544,7 +544,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>yes sign me up</t>
+          <t>Yes sign me up</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -566,7 +566,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>text is better, im at work days</t>
+          <t>Text is better, I'm at work days</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">

</xml_diff>